<commit_message>
Recalibrate OHP, row, and shrug loads from AMRAP tests.
Measured 40x12 (OHP), 40x18 (row), and 50x13 (shrug) at RPE 10 showed the default 80 kg OHP and DL-based accessory percents were far too heavy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/16week-training-program.xlsx
+++ b/16week-training-program.xlsx
@@ -792,10 +792,10 @@
         <v>12</v>
       </c>
       <c r="K7" t="str">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="L7">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="M7" t="str">
         <v/>
@@ -904,10 +904,10 @@
         <v>8</v>
       </c>
       <c r="K9" t="str">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="L9">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1016,10 +1016,10 @@
         <v>12</v>
       </c>
       <c r="K11" t="str">
-        <v>45</v>
+        <v>32.5</v>
       </c>
       <c r="L11">
-        <v>45</v>
+        <v>32.5</v>
       </c>
       <c r="M11" t="str">
         <v/>
@@ -1072,10 +1072,10 @@
         <v>15</v>
       </c>
       <c r="K12" t="str">
-        <v>122.5</v>
+        <v>47.5</v>
       </c>
       <c r="L12">
-        <v>122.5</v>
+        <v>47.5</v>
       </c>
       <c r="M12" t="str">
         <v/>
@@ -1128,10 +1128,10 @@
         <v>8</v>
       </c>
       <c r="K13" t="str">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="L13">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="M13">
         <v>67.5</v>
@@ -1688,10 +1688,10 @@
         <v>12</v>
       </c>
       <c r="K23" t="str">
-        <v>122.5</v>
+        <v>47.5</v>
       </c>
       <c r="L23">
-        <v>122.5</v>
+        <v>47.5</v>
       </c>
       <c r="M23" t="str">
         <v/>
@@ -2024,10 +2024,10 @@
         <v>12</v>
       </c>
       <c r="K29" t="str">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="L29">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="M29" t="str">
         <v/>
@@ -2360,10 +2360,10 @@
         <v>12</v>
       </c>
       <c r="K35" t="str">
-        <v>132.5</v>
+        <v>52.5</v>
       </c>
       <c r="L35">
-        <v>132.5</v>
+        <v>52.5</v>
       </c>
       <c r="M35" t="str">
         <v/>
@@ -2472,10 +2472,10 @@
         <v>8</v>
       </c>
       <c r="K37" t="str">
-        <v>72.5</v>
+        <v>52.5</v>
       </c>
       <c r="L37">
-        <v>72.5</v>
+        <v>52.5</v>
       </c>
       <c r="M37" t="str">
         <v/>
@@ -2584,10 +2584,10 @@
         <v>12</v>
       </c>
       <c r="K39" t="str">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="L39">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="M39" t="str">
         <v/>
@@ -2640,10 +2640,10 @@
         <v>15</v>
       </c>
       <c r="K40" t="str">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="L40">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="M40" t="str">
         <v/>
@@ -2696,10 +2696,10 @@
         <v>8</v>
       </c>
       <c r="K41" t="str">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="L41">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="M41">
         <v>70</v>
@@ -3256,10 +3256,10 @@
         <v>12</v>
       </c>
       <c r="K51" t="str">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="L51">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="M51" t="str">
         <v/>
@@ -3592,10 +3592,10 @@
         <v>12</v>
       </c>
       <c r="K57" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L57">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M57" t="str">
         <v/>
@@ -3928,10 +3928,10 @@
         <v>12</v>
       </c>
       <c r="K63" t="str">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="L63">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="M63" t="str">
         <v/>
@@ -4040,10 +4040,10 @@
         <v>8</v>
       </c>
       <c r="K65" t="str">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="L65">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="M65" t="str">
         <v/>
@@ -4152,10 +4152,10 @@
         <v>12</v>
       </c>
       <c r="K67" t="str">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="L67">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M67" t="str">
         <v/>
@@ -4208,10 +4208,10 @@
         <v>15</v>
       </c>
       <c r="K68" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L68">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M68" t="str">
         <v/>
@@ -4264,10 +4264,10 @@
         <v>6</v>
       </c>
       <c r="K69" t="str">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="L69">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="M69">
         <v>75</v>
@@ -4824,10 +4824,10 @@
         <v>12</v>
       </c>
       <c r="K79" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L79">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M79" t="str">
         <v/>
@@ -5160,10 +5160,10 @@
         <v>12</v>
       </c>
       <c r="K85" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L85">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M85" t="str">
         <v/>
@@ -5496,10 +5496,10 @@
         <v>12</v>
       </c>
       <c r="K91" t="str">
-        <v>115</v>
+        <v>47.5</v>
       </c>
       <c r="L91">
-        <v>115</v>
+        <v>47.5</v>
       </c>
       <c r="M91" t="str">
         <v/>
@@ -5608,10 +5608,10 @@
         <v>8</v>
       </c>
       <c r="K93" t="str">
-        <v>65</v>
+        <v>47.5</v>
       </c>
       <c r="L93">
-        <v>65</v>
+        <v>47.5</v>
       </c>
       <c r="M93" t="str">
         <v/>
@@ -5720,10 +5720,10 @@
         <v>12</v>
       </c>
       <c r="K95" t="str">
-        <v>42.5</v>
+        <v>32.5</v>
       </c>
       <c r="L95">
-        <v>42.5</v>
+        <v>32.5</v>
       </c>
       <c r="M95" t="str">
         <v/>
@@ -5776,10 +5776,10 @@
         <v>15</v>
       </c>
       <c r="K96" t="str">
-        <v>107.5</v>
+        <v>45</v>
       </c>
       <c r="L96">
-        <v>107.5</v>
+        <v>45</v>
       </c>
       <c r="M96" t="str">
         <v/>
@@ -5832,10 +5832,10 @@
         <v>5</v>
       </c>
       <c r="K97" t="str">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="L97">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="M97">
         <v>60</v>
@@ -6392,10 +6392,10 @@
         <v>12</v>
       </c>
       <c r="K107" t="str">
-        <v>107.5</v>
+        <v>45</v>
       </c>
       <c r="L107">
-        <v>107.5</v>
+        <v>45</v>
       </c>
       <c r="M107" t="str">
         <v/>
@@ -6728,10 +6728,10 @@
         <v>12</v>
       </c>
       <c r="K113" t="str">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="L113">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="M113" t="str">
         <v/>
@@ -7064,10 +7064,10 @@
         <v>10-12</v>
       </c>
       <c r="K119" t="str">
-        <v>132.5</v>
+        <v>52.5</v>
       </c>
       <c r="L119">
-        <v>132.5</v>
+        <v>52.5</v>
       </c>
       <c r="M119" t="str">
         <v/>
@@ -7176,10 +7176,10 @@
         <v>8</v>
       </c>
       <c r="K121" t="str">
-        <v>72.5</v>
+        <v>52.5</v>
       </c>
       <c r="L121">
-        <v>72.5</v>
+        <v>52.5</v>
       </c>
       <c r="M121" t="str">
         <v/>
@@ -7288,10 +7288,10 @@
         <v>10</v>
       </c>
       <c r="K123" t="str">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="L123">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="M123" t="str">
         <v/>
@@ -7344,10 +7344,10 @@
         <v>12</v>
       </c>
       <c r="K124" t="str">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="L124">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="M124" t="str">
         <v/>
@@ -7400,10 +7400,10 @@
         <v>6</v>
       </c>
       <c r="K125" t="str">
-        <v>57.5</v>
+        <v>42.5</v>
       </c>
       <c r="L125">
-        <v>57.5</v>
+        <v>42.5</v>
       </c>
       <c r="M125">
         <v>72.5</v>
@@ -7960,10 +7960,10 @@
         <v>12</v>
       </c>
       <c r="K135" t="str">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="L135">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="M135" t="str">
         <v/>
@@ -8296,10 +8296,10 @@
         <v>12</v>
       </c>
       <c r="K141" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L141">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M141" t="str">
         <v/>
@@ -8632,10 +8632,10 @@
         <v>10-12</v>
       </c>
       <c r="K147" t="str">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="L147">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="M147" t="str">
         <v/>
@@ -8744,10 +8744,10 @@
         <v>8</v>
       </c>
       <c r="K149" t="str">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="L149">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="M149" t="str">
         <v/>
@@ -8856,10 +8856,10 @@
         <v>10</v>
       </c>
       <c r="K151" t="str">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="L151">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M151" t="str">
         <v/>
@@ -8912,10 +8912,10 @@
         <v>12</v>
       </c>
       <c r="K152" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L152">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M152" t="str">
         <v/>
@@ -8968,10 +8968,10 @@
         <v>6</v>
       </c>
       <c r="K153" t="str">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="L153">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="M153">
         <v>75</v>
@@ -9528,10 +9528,10 @@
         <v>12</v>
       </c>
       <c r="K163" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L163">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M163" t="str">
         <v/>
@@ -9864,10 +9864,10 @@
         <v>12</v>
       </c>
       <c r="K169" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L169">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M169" t="str">
         <v/>
@@ -10200,10 +10200,10 @@
         <v>10-12</v>
       </c>
       <c r="K175" t="str">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="L175">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="M175" t="str">
         <v/>
@@ -10312,10 +10312,10 @@
         <v>8</v>
       </c>
       <c r="K177" t="str">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="L177">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="M177" t="str">
         <v/>
@@ -10424,10 +10424,10 @@
         <v>10</v>
       </c>
       <c r="K179" t="str">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="L179">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="M179" t="str">
         <v/>
@@ -10480,10 +10480,10 @@
         <v>12</v>
       </c>
       <c r="K180" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L180">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M180" t="str">
         <v/>
@@ -10536,10 +10536,10 @@
         <v>5</v>
       </c>
       <c r="K181" t="str">
-        <v>62.5</v>
+        <v>47.5</v>
       </c>
       <c r="L181">
-        <v>62.5</v>
+        <v>47.5</v>
       </c>
       <c r="M181">
         <v>77.5</v>
@@ -11096,10 +11096,10 @@
         <v>12</v>
       </c>
       <c r="K191" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L191">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M191" t="str">
         <v/>
@@ -11432,10 +11432,10 @@
         <v>12</v>
       </c>
       <c r="K197" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L197">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M197" t="str">
         <v/>
@@ -11768,10 +11768,10 @@
         <v>10-12</v>
       </c>
       <c r="K203" t="str">
-        <v>117.5</v>
+        <v>50</v>
       </c>
       <c r="L203">
-        <v>117.5</v>
+        <v>50</v>
       </c>
       <c r="M203" t="str">
         <v/>
@@ -11880,10 +11880,10 @@
         <v>8</v>
       </c>
       <c r="K205" t="str">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="L205">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="M205" t="str">
         <v/>
@@ -11992,10 +11992,10 @@
         <v>10</v>
       </c>
       <c r="K207" t="str">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="L207">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="M207" t="str">
         <v/>
@@ -12048,10 +12048,10 @@
         <v>12</v>
       </c>
       <c r="K208" t="str">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="L208">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="M208" t="str">
         <v/>
@@ -12104,10 +12104,10 @@
         <v>5</v>
       </c>
       <c r="K209" t="str">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="L209">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M209">
         <v>62.5</v>
@@ -12664,10 +12664,10 @@
         <v>12</v>
       </c>
       <c r="K219" t="str">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="L219">
-        <v>110</v>
+        <v>47.5</v>
       </c>
       <c r="M219" t="str">
         <v/>
@@ -13000,10 +13000,10 @@
         <v>12</v>
       </c>
       <c r="K225" t="str">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="L225">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="M225" t="str">
         <v/>
@@ -13336,10 +13336,10 @@
         <v>10</v>
       </c>
       <c r="K231" t="str">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="L231">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="M231" t="str">
         <v/>
@@ -13448,10 +13448,10 @@
         <v>6-8</v>
       </c>
       <c r="K233" t="str">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="L233">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="M233" t="str">
         <v/>
@@ -13560,10 +13560,10 @@
         <v>10</v>
       </c>
       <c r="K235" t="str">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="L235">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M235" t="str">
         <v/>
@@ -13616,10 +13616,10 @@
         <v>12</v>
       </c>
       <c r="K236" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L236">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M236" t="str">
         <v/>
@@ -13672,10 +13672,10 @@
         <v>5</v>
       </c>
       <c r="K237" t="str">
-        <v>62.5</v>
+        <v>47.5</v>
       </c>
       <c r="L237">
-        <v>62.5</v>
+        <v>47.5</v>
       </c>
       <c r="M237">
         <v>77.5</v>
@@ -14232,10 +14232,10 @@
         <v>10</v>
       </c>
       <c r="K247" t="str">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="L247">
-        <v>127.5</v>
+        <v>52.5</v>
       </c>
       <c r="M247" t="str">
         <v/>
@@ -14568,10 +14568,10 @@
         <v>10</v>
       </c>
       <c r="K253" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L253">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M253" t="str">
         <v/>
@@ -14904,10 +14904,10 @@
         <v>10</v>
       </c>
       <c r="K259" t="str">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="L259">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="M259" t="str">
         <v/>
@@ -15016,10 +15016,10 @@
         <v>6-8</v>
       </c>
       <c r="K261" t="str">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="L261">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="M261" t="str">
         <v/>
@@ -15128,10 +15128,10 @@
         <v>10</v>
       </c>
       <c r="K263" t="str">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="L263">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="M263" t="str">
         <v/>
@@ -15184,10 +15184,10 @@
         <v>12</v>
       </c>
       <c r="K264" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L264">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M264" t="str">
         <v/>
@@ -15240,10 +15240,10 @@
         <v>4</v>
       </c>
       <c r="K265" t="str">
-        <v>65</v>
+        <v>47.5</v>
       </c>
       <c r="L265">
-        <v>65</v>
+        <v>47.5</v>
       </c>
       <c r="M265">
         <v>80</v>
@@ -15800,10 +15800,10 @@
         <v>10</v>
       </c>
       <c r="K275" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L275">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M275" t="str">
         <v/>
@@ -16136,10 +16136,10 @@
         <v>10</v>
       </c>
       <c r="K281" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L281">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M281" t="str">
         <v/>
@@ -16472,10 +16472,10 @@
         <v>10</v>
       </c>
       <c r="K287" t="str">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="L287">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="M287" t="str">
         <v/>
@@ -16584,10 +16584,10 @@
         <v>6-8</v>
       </c>
       <c r="K289" t="str">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="L289">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="M289" t="str">
         <v/>
@@ -16696,10 +16696,10 @@
         <v>10</v>
       </c>
       <c r="K291" t="str">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="L291">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="M291" t="str">
         <v/>
@@ -16752,10 +16752,10 @@
         <v>12</v>
       </c>
       <c r="K292" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L292">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M292" t="str">
         <v/>
@@ -16808,10 +16808,10 @@
         <v>3</v>
       </c>
       <c r="K293" t="str">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="L293">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="M293">
         <v>82.5</v>
@@ -17368,10 +17368,10 @@
         <v>10</v>
       </c>
       <c r="K303" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L303">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M303" t="str">
         <v/>
@@ -17704,10 +17704,10 @@
         <v>10</v>
       </c>
       <c r="K309" t="str">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L309">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="M309" t="str">
         <v/>
@@ -18040,10 +18040,10 @@
         <v>10</v>
       </c>
       <c r="K315" t="str">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="L315">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="M315" t="str">
         <v/>
@@ -18152,10 +18152,10 @@
         <v>6-8</v>
       </c>
       <c r="K317" t="str">
-        <v>67.5</v>
+        <v>50</v>
       </c>
       <c r="L317">
-        <v>67.5</v>
+        <v>50</v>
       </c>
       <c r="M317" t="str">
         <v/>
@@ -18264,10 +18264,10 @@
         <v>10</v>
       </c>
       <c r="K319" t="str">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="L319">
-        <v>47.5</v>
+        <v>35</v>
       </c>
       <c r="M319" t="str">
         <v/>
@@ -18320,10 +18320,10 @@
         <v>12</v>
       </c>
       <c r="K320" t="str">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="L320">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="M320" t="str">
         <v/>
@@ -18376,10 +18376,10 @@
         <v>4</v>
       </c>
       <c r="K321" t="str">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="L321">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="M321">
         <v>65</v>
@@ -18936,10 +18936,10 @@
         <v>10</v>
       </c>
       <c r="K331" t="str">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="L331">
-        <v>112.5</v>
+        <v>50</v>
       </c>
       <c r="M331" t="str">
         <v/>
@@ -19272,10 +19272,10 @@
         <v>10</v>
       </c>
       <c r="K337" t="str">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="L337">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="M337" t="str">
         <v/>
@@ -19608,10 +19608,10 @@
         <v>10</v>
       </c>
       <c r="K343" t="str">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="L343">
-        <v>137.5</v>
+        <v>57.5</v>
       </c>
       <c r="M343" t="str">
         <v/>
@@ -19720,10 +19720,10 @@
         <v>6</v>
       </c>
       <c r="K345" t="str">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="L345">
-        <v>77.5</v>
+        <v>57.5</v>
       </c>
       <c r="M345" t="str">
         <v/>
@@ -19832,10 +19832,10 @@
         <v>10</v>
       </c>
       <c r="K347" t="str">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="L347">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="M347" t="str">
         <v/>
@@ -19888,10 +19888,10 @@
         <v>10</v>
       </c>
       <c r="K348" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L348">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M348" t="str">
         <v/>
@@ -19944,10 +19944,10 @@
         <v>3</v>
       </c>
       <c r="K349" t="str">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="L349">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="M349">
         <v>82.5</v>
@@ -20504,10 +20504,10 @@
         <v>10</v>
       </c>
       <c r="K359" t="str">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="L359">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="M359" t="str">
         <v/>
@@ -20840,10 +20840,10 @@
         <v>8</v>
       </c>
       <c r="K365" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L365">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M365" t="str">
         <v/>
@@ -21176,10 +21176,10 @@
         <v>10</v>
       </c>
       <c r="K371" t="str">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="L371">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="M371" t="str">
         <v/>
@@ -21288,10 +21288,10 @@
         <v>6</v>
       </c>
       <c r="K373" t="str">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="L373">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="M373" t="str">
         <v/>
@@ -21400,10 +21400,10 @@
         <v>10</v>
       </c>
       <c r="K375" t="str">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="L375">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="M375" t="str">
         <v/>
@@ -21456,10 +21456,10 @@
         <v>10</v>
       </c>
       <c r="K376" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L376">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M376" t="str">
         <v/>
@@ -21512,10 +21512,10 @@
         <v>3</v>
       </c>
       <c r="K377" t="str">
-        <v>67.5</v>
+        <v>50</v>
       </c>
       <c r="L377">
-        <v>67.5</v>
+        <v>50</v>
       </c>
       <c r="M377">
         <v>85</v>
@@ -22072,10 +22072,10 @@
         <v>10</v>
       </c>
       <c r="K387" t="str">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="L387">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="M387" t="str">
         <v/>
@@ -22408,10 +22408,10 @@
         <v>8</v>
       </c>
       <c r="K393" t="str">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L393">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="M393" t="str">
         <v/>
@@ -22744,10 +22744,10 @@
         <v>10</v>
       </c>
       <c r="K399" t="str">
-        <v>142.5</v>
+        <v>62.5</v>
       </c>
       <c r="L399">
-        <v>142.5</v>
+        <v>62.5</v>
       </c>
       <c r="M399" t="str">
         <v/>
@@ -22856,10 +22856,10 @@
         <v>6</v>
       </c>
       <c r="K401" t="str">
-        <v>82.5</v>
+        <v>62.5</v>
       </c>
       <c r="L401">
-        <v>82.5</v>
+        <v>62.5</v>
       </c>
       <c r="M401" t="str">
         <v/>
@@ -22968,10 +22968,10 @@
         <v>10</v>
       </c>
       <c r="K403" t="str">
-        <v>57.5</v>
+        <v>45</v>
       </c>
       <c r="L403">
-        <v>57.5</v>
+        <v>45</v>
       </c>
       <c r="M403" t="str">
         <v/>
@@ -23024,10 +23024,10 @@
         <v>10</v>
       </c>
       <c r="K404" t="str">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L404">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="M404" t="str">
         <v/>
@@ -23080,10 +23080,10 @@
         <v>2</v>
       </c>
       <c r="K405" t="str">
-        <v>70</v>
+        <v>52.5</v>
       </c>
       <c r="L405">
-        <v>70</v>
+        <v>52.5</v>
       </c>
       <c r="M405">
         <v>87.5</v>
@@ -23640,10 +23640,10 @@
         <v>10</v>
       </c>
       <c r="K415" t="str">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L415">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="M415" t="str">
         <v/>
@@ -23976,10 +23976,10 @@
         <v>8</v>
       </c>
       <c r="K421" t="str">
-        <v>137.5</v>
+        <v>62.5</v>
       </c>
       <c r="L421">
-        <v>137.5</v>
+        <v>62.5</v>
       </c>
       <c r="M421" t="str">
         <v/>
@@ -24312,10 +24312,10 @@
         <v>10</v>
       </c>
       <c r="K427" t="str">
-        <v>120</v>
+        <v>52.5</v>
       </c>
       <c r="L427">
-        <v>120</v>
+        <v>52.5</v>
       </c>
       <c r="M427" t="str">
         <v/>
@@ -24424,10 +24424,10 @@
         <v>6</v>
       </c>
       <c r="K429" t="str">
-        <v>70</v>
+        <v>52.5</v>
       </c>
       <c r="L429">
-        <v>70</v>
+        <v>52.5</v>
       </c>
       <c r="M429" t="str">
         <v/>
@@ -24536,10 +24536,10 @@
         <v>10</v>
       </c>
       <c r="K431" t="str">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="L431">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="M431" t="str">
         <v/>
@@ -24592,10 +24592,10 @@
         <v>10</v>
       </c>
       <c r="K432" t="str">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="L432">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="M432" t="str">
         <v/>
@@ -24648,10 +24648,10 @@
         <v>4</v>
       </c>
       <c r="K433" t="str">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="L433">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="M433">
         <v>65</v>
@@ -25208,10 +25208,10 @@
         <v>10</v>
       </c>
       <c r="K443" t="str">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="L443">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="M443" t="str">
         <v/>
@@ -25544,10 +25544,10 @@
         <v>8</v>
       </c>
       <c r="K449" t="str">
-        <v>117.5</v>
+        <v>52.5</v>
       </c>
       <c r="L449">
-        <v>117.5</v>
+        <v>52.5</v>
       </c>
       <c r="M449" t="str">
         <v/>
@@ -27230,7 +27230,7 @@
         <v>オーバーヘッドプレス</v>
       </c>
       <c r="B5">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C5" t="str">
         <v>未計測なら推定。RPEで修正</v>

</xml_diff>